<commit_message>
add dates and fix whitespace
</commit_message>
<xml_diff>
--- a/data/master-sheet updated.xlsx
+++ b/data/master-sheet updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jon/Documents/projects/clio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0802C7F7-97D1-FA45-93A5-7C2A45E8DA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{687420B1-4DD7-524E-A601-105395D57684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="760" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>address</t>
   </si>
@@ -1150,6 +1150,9 @@
   </si>
   <si>
     <t>application_type</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -1707,7 +1710,7 @@
     <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1737,6 +1740,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2089,6 +2093,7 @@
     <col min="3" max="3" width="21.33203125" customWidth="1"/>
     <col min="4" max="4" width="45.33203125" customWidth="1"/>
     <col min="5" max="5" width="33.1640625" customWidth="1"/>
+    <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2108,7 +2113,9 @@
       <c r="E1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="2"/>
+      <c r="F1" s="2" t="s">
+        <v>80</v>
+      </c>
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -2127,6 +2134,9 @@
       <c r="E2" t="s">
         <v>50</v>
       </c>
+      <c r="F2" s="11">
+        <v>43906</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -2144,6 +2154,9 @@
       <c r="E3" t="s">
         <v>51</v>
       </c>
+      <c r="F3" s="11">
+        <v>43906</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -2161,6 +2174,9 @@
       <c r="E4" t="s">
         <v>51</v>
       </c>
+      <c r="F4" s="11">
+        <v>45196</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -2178,6 +2194,9 @@
       <c r="E5" t="s">
         <v>50</v>
       </c>
+      <c r="F5" s="11">
+        <v>45196</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -2195,6 +2214,9 @@
       <c r="E6" t="s">
         <v>49</v>
       </c>
+      <c r="F6" s="11">
+        <v>45411</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -2212,6 +2234,9 @@
       <c r="E7" t="s">
         <v>49</v>
       </c>
+      <c r="F7" s="11">
+        <v>45546</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -2229,6 +2254,9 @@
       <c r="E8" t="s">
         <v>47</v>
       </c>
+      <c r="F8" s="11">
+        <v>45742</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -2246,6 +2274,9 @@
       <c r="E9" t="s">
         <v>47</v>
       </c>
+      <c r="F9" s="11">
+        <v>45733</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -2263,6 +2294,9 @@
       <c r="E10" t="s">
         <v>45</v>
       </c>
+      <c r="F10" s="11">
+        <v>45637</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -2280,6 +2314,9 @@
       <c r="E11" t="s">
         <v>47</v>
       </c>
+      <c r="F11" s="11">
+        <v>45615</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -2297,6 +2334,9 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
+      <c r="F12" s="11">
+        <v>45212</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -2314,6 +2354,9 @@
       <c r="E13" t="s">
         <v>48</v>
       </c>
+      <c r="F13" s="11">
+        <v>45139</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -2331,6 +2374,9 @@
       <c r="E14" t="s">
         <v>47</v>
       </c>
+      <c r="F14" s="11">
+        <v>45138</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -2348,6 +2394,9 @@
       <c r="E15" t="s">
         <v>45</v>
       </c>
+      <c r="F15" s="11">
+        <v>44970</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -2364,6 +2413,9 @@
       </c>
       <c r="E16" t="s">
         <v>46</v>
+      </c>
+      <c r="F16" s="11">
+        <v>44344</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.25">
@@ -2420,7 +2472,9 @@
       <c r="E19" t="s">
         <v>56</v>
       </c>
-      <c r="F19" s="4"/>
+      <c r="F19" s="5">
+        <v>45458</v>
+      </c>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:7" ht="100" thickBot="1" x14ac:dyDescent="0.25">
@@ -2439,7 +2493,9 @@
       <c r="E20" t="s">
         <v>56</v>
       </c>
-      <c r="F20" s="4"/>
+      <c r="F20" s="5">
+        <v>45580</v>
+      </c>
       <c r="G20" s="5"/>
     </row>
     <row r="21" spans="1:7" ht="399" thickBot="1" x14ac:dyDescent="0.25">
@@ -2458,6 +2514,9 @@
       <c r="E21" s="7" t="s">
         <v>78</v>
       </c>
+      <c r="F21" s="11">
+        <v>45089</v>
+      </c>
     </row>
     <row r="22" spans="1:7" ht="211" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
@@ -2475,6 +2534,9 @@
       <c r="E22" s="7" t="s">
         <v>78</v>
       </c>
+      <c r="F22" s="11">
+        <v>44942</v>
+      </c>
     </row>
     <row r="23" spans="1:7" ht="225" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
@@ -2492,6 +2554,9 @@
       <c r="E23" t="s">
         <v>78</v>
       </c>
+      <c r="F23" s="11">
+        <v>44998</v>
+      </c>
     </row>
     <row r="24" spans="1:7" ht="315" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
@@ -2508,6 +2573,9 @@
       </c>
       <c r="E24" s="7" t="s">
         <v>78</v>
+      </c>
+      <c r="F24" s="11">
+        <v>45113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>